<commit_message>
assembly and bom progress
</commit_message>
<xml_diff>
--- a/other/vacuum_instrumentation_bundle_v2/bom/BOM (version 1).xlsx
+++ b/other/vacuum_instrumentation_bundle_v2/bom/BOM (version 1).xlsx
@@ -8,20 +8,34 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aiden\Documents\GitHub\coldex-instrumentation\other\vacuum_instrumentation_bundle_v2\bom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E4DBCDE-0CD4-47A0-AD5D-4F4310BEAC5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{191951C3-3B69-401C-89FA-9664CB749EFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32250" yWindow="0" windowWidth="19350" windowHeight="21000" activeTab="1" xr2:uid="{64365B26-9AB1-4F2A-B9FA-C5EB43087255}"/>
+    <workbookView xWindow="25800" yWindow="0" windowWidth="25800" windowHeight="21000" activeTab="1" xr2:uid="{64365B26-9AB1-4F2A-B9FA-C5EB43087255}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
     <sheet name="BOM_revised" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="179">
   <si>
     <t>Group</t>
   </si>
@@ -551,6 +565,15 @@
   </si>
   <si>
     <t>ea (10 pack)</t>
+  </si>
+  <si>
+    <t>Nice to have items</t>
+  </si>
+  <si>
+    <t>80/20 handle for carrying</t>
+  </si>
+  <si>
+    <t>80/20 cable tie mounts</t>
   </si>
 </sst>
 </file>
@@ -1063,7 +1086,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -1081,6 +1104,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -3189,4 +3214,32 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId22"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53FFDAE8-D232-4FAD-9028-6E53C5768A44}">
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="45.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>178</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>